<commit_message>
Change table colors to teal and gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qf3WFgE5dEcxE39muo45t
</commit_message>
<xml_diff>
--- a/جدول_أسعار_الوحدات.xlsx
+++ b/جدول_أسعار_الوحدات.xlsx
@@ -55,17 +55,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="000F4C45"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
+        <fgColor rgb="00B08D57"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00F5EFE3"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,16 +84,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="008EA9DB"/>
+        <color rgb="00C9B48A"/>
       </left>
       <right style="thin">
-        <color rgb="008EA9DB"/>
+        <color rgb="00C9B48A"/>
       </right>
       <top style="thin">
-        <color rgb="008EA9DB"/>
+        <color rgb="00C9B48A"/>
       </top>
       <bottom style="thin">
-        <color rgb="008EA9DB"/>
+        <color rgb="00C9B48A"/>
       </bottom>
     </border>
   </borders>

</xml_diff>